<commit_message>
Snapshot current DongLanpec code and required resources
Capture the local source, CAD and report templates, DLL dependencies, and static MySQL distribution as of 2026-10-15. Exclude local login settings, runtime databases, caches, and build output.
</commit_message>
<xml_diff>
--- a/modules/chanpinguanli/条件输入数据表.xlsx
+++ b/modules/chanpinguanli/条件输入数据表.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9060" activeTab="2"/>
+    <workbookView windowWidth="22188" windowHeight="9060" firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="产品标准" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="173">
   <si>
     <t>规范/标准序号</t>
   </si>
@@ -165,42 +165,48 @@
     <t>mm</t>
   </si>
   <si>
+    <t>介质名称</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>设计压力*</t>
+  </si>
+  <si>
+    <t>Mpa</t>
+  </si>
+  <si>
     <t>介质特性（毒性危害程度）</t>
   </si>
   <si>
-    <t>设计压力*</t>
-  </si>
-  <si>
-    <t>Mpa</t>
+    <t>设计温度（最高）*</t>
+  </si>
+  <si>
+    <t>℃</t>
   </si>
   <si>
     <t>介质特性（爆炸危险程度）</t>
   </si>
   <si>
-    <t>设计温度（最高）*</t>
-  </si>
-  <si>
-    <t>℃</t>
+    <t>工作压力</t>
+  </si>
+  <si>
+    <t>MPa</t>
   </si>
   <si>
     <t>介质特性（是否液化气体）</t>
   </si>
   <si>
-    <t>工作压力</t>
-  </si>
-  <si>
-    <t>MPa</t>
-  </si>
-  <si>
     <t>工作温度（入口）</t>
   </si>
   <si>
+    <t>工作温度（出口）</t>
+  </si>
+  <si>
     <t xml:space="preserve">设计压力* </t>
   </si>
   <si>
-    <t>工作温度（出口）</t>
-  </si>
-  <si>
     <t>最高允许工作压力</t>
   </si>
   <si>
@@ -219,16 +225,19 @@
     <t>13</t>
   </si>
   <si>
+    <t>14</t>
+  </si>
+  <si>
     <t>最低设计温度</t>
   </si>
   <si>
-    <t>14</t>
+    <t>15</t>
   </si>
   <si>
     <t>腐蚀裕量*</t>
   </si>
   <si>
-    <t>15</t>
+    <t>16</t>
   </si>
   <si>
     <t>焊接接头系数*</t>
@@ -237,25 +246,25 @@
     <t>1.0</t>
   </si>
   <si>
-    <t>16</t>
+    <t>17</t>
   </si>
   <si>
     <t>液柱静压力</t>
   </si>
   <si>
-    <t>17</t>
+    <t>18</t>
   </si>
   <si>
     <t>介质（组分）</t>
   </si>
   <si>
-    <t>18</t>
+    <t>19</t>
   </si>
   <si>
     <t>介质（相态）</t>
   </si>
   <si>
-    <t>19</t>
+    <t>20</t>
   </si>
   <si>
     <t>介质密度</t>
@@ -264,7 +273,7 @@
     <t>kg/m³</t>
   </si>
   <si>
-    <t>20</t>
+    <t>21</t>
   </si>
   <si>
     <t>介质入口流速</t>
@@ -273,16 +282,13 @@
     <t>m/s</t>
   </si>
   <si>
-    <t>21</t>
+    <t>22</t>
   </si>
   <si>
     <t>超压泄放装置</t>
   </si>
   <si>
     <t>工艺系统考虑</t>
-  </si>
-  <si>
-    <t>22</t>
   </si>
   <si>
     <t>耐压试验类型*</t>
@@ -946,7 +952,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="27">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -1174,19 +1180,6 @@
         <color auto="1"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1326,7 +1319,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1338,34 +1331,34 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="26" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1450,7 +1443,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1537,13 +1530,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1884,11 +1874,11 @@
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="14" style="35" customWidth="1"/>
-    <col min="2" max="2" width="17.0925925925926" style="36" customWidth="1"/>
-    <col min="3" max="3" width="38.0925925925926" style="36" customWidth="1"/>
-    <col min="4" max="6" width="9" style="36" customWidth="1"/>
-    <col min="7" max="16384" width="9" style="36"/>
+    <col min="1" max="1" width="14" style="34" customWidth="1"/>
+    <col min="2" max="2" width="17.0925925925926" style="35" customWidth="1"/>
+    <col min="3" max="3" width="38.0925925925926" style="35" customWidth="1"/>
+    <col min="4" max="6" width="9" style="35" customWidth="1"/>
+    <col min="7" max="16384" width="9" style="35"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.15" spans="1:3">
@@ -1903,121 +1893,121 @@
       </c>
     </row>
     <row r="2" ht="17.4" spans="1:3">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="39" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="36" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" ht="17.4" spans="1:3">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="40" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="38" t="s">
+      <c r="C3" s="37" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="4" ht="17.4" spans="1:3">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="40" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="38"/>
+      <c r="C4" s="37"/>
     </row>
     <row r="5" ht="17.4" spans="1:3">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="40" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="38" t="s">
+      <c r="C5" s="37" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" ht="17.4" spans="1:3">
-      <c r="A6" s="41" t="s">
+      <c r="A6" s="40" t="s">
         <v>14</v>
       </c>
       <c r="B6" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="38" t="s">
+      <c r="C6" s="37" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="7" ht="17.4" spans="1:3">
-      <c r="A7" s="41" t="s">
+      <c r="A7" s="40" t="s">
         <v>17</v>
       </c>
       <c r="B7" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="38" t="s">
+      <c r="C7" s="37" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="8" ht="17.4" spans="1:3">
-      <c r="A8" s="41" t="s">
+      <c r="A8" s="40" t="s">
         <v>20</v>
       </c>
       <c r="B8" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="38" t="s">
+      <c r="C8" s="37" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="9" ht="17.4" spans="1:3">
-      <c r="A9" s="41" t="s">
+      <c r="A9" s="40" t="s">
         <v>23</v>
       </c>
       <c r="B9" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="38" t="s">
+      <c r="C9" s="37" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" ht="17.4" spans="1:3">
-      <c r="A10" s="41" t="s">
+      <c r="A10" s="40" t="s">
         <v>26</v>
       </c>
       <c r="B10" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="38" t="s">
+      <c r="C10" s="37" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="11" ht="17.4" spans="1:3">
-      <c r="A11" s="41" t="s">
+      <c r="A11" s="40" t="s">
         <v>29</v>
       </c>
       <c r="B11" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="38" t="s">
+      <c r="C11" s="37" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="12" ht="18.15" spans="1:3">
-      <c r="A12" s="42" t="s">
+      <c r="A12" s="41" t="s">
         <v>32</v>
       </c>
       <c r="B12" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="C12" s="39" t="s">
+      <c r="C12" s="38" t="s">
         <v>34</v>
       </c>
     </row>
@@ -2031,11 +2021,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.4"/>
   <cols>
     <col min="1" max="1" width="9" style="15" customWidth="1"/>
-    <col min="2" max="2" width="25.3611111111111" style="14" customWidth="1"/>
+    <col min="2" max="2" width="30.6666666666667" style="14" customWidth="1"/>
     <col min="3" max="3" width="9.90740740740741" style="15" customWidth="1"/>
     <col min="4" max="5" width="13.7222222222222" style="15" customWidth="1"/>
     <col min="6" max="6" width="9" style="14" customWidth="1"/>
@@ -2080,7 +2070,7 @@
       <c r="L1" s="8"/>
     </row>
     <row r="2" spans="1:12">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="39" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="20" t="s">
@@ -2107,20 +2097,22 @@
       </c>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
+      <c r="C3" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" s="20"/>
       <c r="E3" s="25"/>
       <c r="G3" s="24" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I3" s="24"/>
       <c r="J3" s="24"/>
@@ -2128,20 +2120,20 @@
       <c r="L3" s="24"/>
     </row>
     <row r="4" spans="1:12">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="40" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="24" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C4" s="8"/>
       <c r="D4" s="8"/>
       <c r="E4" s="25"/>
       <c r="G4" s="24" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I4" s="24"/>
       <c r="J4" s="24"/>
@@ -2149,20 +2141,20 @@
       <c r="L4" s="24"/>
     </row>
     <row r="5" spans="1:12">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="32" t="s">
-        <v>50</v>
-      </c>
-      <c r="C5" s="33"/>
+      <c r="B5" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5" s="8"/>
       <c r="D5" s="8"/>
       <c r="E5" s="25"/>
       <c r="G5" s="24" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I5" s="24"/>
       <c r="J5" s="24"/>
@@ -2170,22 +2162,20 @@
       <c r="L5" s="24"/>
     </row>
     <row r="6" spans="1:12">
-      <c r="A6" s="41" t="s">
+      <c r="A6" s="40" t="s">
         <v>14</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>52</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="C6" s="32"/>
       <c r="D6" s="8"/>
       <c r="E6" s="25"/>
       <c r="G6" s="24" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I6" s="24"/>
       <c r="J6" s="24"/>
@@ -2193,22 +2183,22 @@
       <c r="L6" s="24"/>
     </row>
     <row r="7" spans="1:12">
-      <c r="A7" s="41" t="s">
+      <c r="A7" s="40" t="s">
         <v>17</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D7" s="8"/>
       <c r="E7" s="25"/>
       <c r="G7" s="24" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I7" s="24"/>
       <c r="J7" s="24"/>
@@ -2216,22 +2206,22 @@
       <c r="L7" s="24"/>
     </row>
     <row r="8" spans="1:12">
-      <c r="A8" s="41" t="s">
+      <c r="A8" s="40" t="s">
         <v>20</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="25"/>
       <c r="G8" s="24" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I8" s="24"/>
       <c r="J8" s="24"/>
@@ -2239,163 +2229,163 @@
       <c r="L8" s="24"/>
     </row>
     <row r="9" spans="1:12">
-      <c r="A9" s="41" t="s">
+      <c r="A9" s="40" t="s">
         <v>23</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D9" s="8"/>
       <c r="E9" s="25"/>
     </row>
     <row r="10" spans="1:12">
-      <c r="A10" s="41" t="s">
+      <c r="A10" s="40" t="s">
         <v>26</v>
       </c>
       <c r="B10" s="24" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="E10" s="25">
+        <v>53</v>
+      </c>
+      <c r="D10" s="8"/>
+      <c r="E10" s="25"/>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" s="40" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E11" s="25">
         <v>0.05</v>
       </c>
     </row>
-    <row r="11" spans="1:12">
-      <c r="A11" s="41" t="s">
-        <v>29</v>
-      </c>
-      <c r="B11" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="C11" s="8" t="s">
+    <row r="12" spans="1:12">
+      <c r="A12" s="40" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="D11" s="8"/>
-      <c r="E11" s="25"/>
-    </row>
-    <row r="12" spans="1:12">
-      <c r="A12" s="41" t="s">
-        <v>32</v>
-      </c>
-      <c r="B12" s="24" t="s">
-        <v>53</v>
-      </c>
       <c r="C12" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D12" s="8"/>
       <c r="E12" s="25"/>
     </row>
     <row r="13" spans="1:12">
-      <c r="A13" s="41" t="s">
-        <v>60</v>
+      <c r="A13" s="40" t="s">
+        <v>62</v>
       </c>
       <c r="B13" s="24" t="s">
         <v>55</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D13" s="8"/>
       <c r="E13" s="25"/>
     </row>
     <row r="14" spans="1:12">
-      <c r="A14" s="41" t="s">
-        <v>61</v>
+      <c r="A14" s="40" t="s">
+        <v>63</v>
       </c>
       <c r="B14" s="24" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D14" s="8"/>
       <c r="E14" s="25"/>
     </row>
     <row r="15" spans="1:12">
-      <c r="A15" s="41" t="s">
-        <v>63</v>
+      <c r="A15" s="40" t="s">
+        <v>64</v>
       </c>
       <c r="B15" s="24" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="D15" s="8"/>
       <c r="E15" s="25"/>
     </row>
     <row r="16" spans="1:12">
-      <c r="A16" s="41" t="s">
-        <v>65</v>
+      <c r="A16" s="40" t="s">
+        <v>66</v>
       </c>
       <c r="B16" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="E16" s="25" t="s">
-        <v>67</v>
-      </c>
+      <c r="C16" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="D16" s="8"/>
+      <c r="E16" s="25"/>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="41" t="s">
+      <c r="A17" s="40" t="s">
         <v>68</v>
       </c>
       <c r="B17" s="24" t="s">
         <v>69</v>
       </c>
       <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="25"/>
+      <c r="D17" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="E17" s="25" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="41" t="s">
-        <v>70</v>
+      <c r="A18" s="40" t="s">
+        <v>71</v>
       </c>
       <c r="B18" s="24" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
       <c r="E18" s="25"/>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="41" t="s">
-        <v>72</v>
+      <c r="A19" s="40" t="s">
+        <v>73</v>
       </c>
       <c r="B19" s="24" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C19" s="8"/>
       <c r="D19" s="8"/>
       <c r="E19" s="25"/>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="41" t="s">
-        <v>74</v>
+      <c r="A20" s="40" t="s">
+        <v>75</v>
       </c>
       <c r="B20" s="24" t="s">
-        <v>75</v>
-      </c>
-      <c r="C20" s="8" t="s">
         <v>76</v>
       </c>
+      <c r="C20" s="8"/>
       <c r="D20" s="8"/>
       <c r="E20" s="25"/>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="41" t="s">
+      <c r="A21" s="40" t="s">
         <v>77</v>
       </c>
       <c r="B21" s="24" t="s">
@@ -2408,22 +2398,20 @@
       <c r="E21" s="25"/>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="41" t="s">
+      <c r="A22" s="40" t="s">
         <v>80</v>
       </c>
       <c r="B22" s="24" t="s">
         <v>81</v>
       </c>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8" t="s">
+      <c r="C22" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="E22" s="25" t="s">
-        <v>82</v>
-      </c>
+      <c r="D22" s="8"/>
+      <c r="E22" s="25"/>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="41" t="s">
+      <c r="A23" s="40" t="s">
         <v>83</v>
       </c>
       <c r="B23" s="24" t="s">
@@ -2444,14 +2432,12 @@
       <c r="B24" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="C24" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="D24" s="8">
-        <v>15</v>
-      </c>
-      <c r="E24" s="34">
-        <v>15</v>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="E24" s="25" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -2459,23 +2445,27 @@
         <v>24</v>
       </c>
       <c r="B25" s="24" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="D25" s="8"/>
-      <c r="E25" s="25"/>
+        <v>50</v>
+      </c>
+      <c r="D25" s="8">
+        <v>15</v>
+      </c>
+      <c r="E25" s="33">
+        <v>15</v>
+      </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="23">
         <v>25</v>
       </c>
       <c r="B26" s="24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D26" s="8"/>
       <c r="E26" s="25"/>
@@ -2485,15 +2475,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="24" t="s">
-        <v>89</v>
-      </c>
-      <c r="C27" s="8"/>
-      <c r="D27" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="E27" s="25" t="s">
-        <v>90</v>
-      </c>
+      <c r="C27" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D27" s="8"/>
+      <c r="E27" s="25"/>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="23">
@@ -2502,9 +2490,7 @@
       <c r="B28" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="C28" s="8" t="s">
-        <v>76</v>
-      </c>
+      <c r="C28" s="8"/>
       <c r="D28" s="8" t="s">
         <v>92</v>
       </c>
@@ -2519,24 +2505,26 @@
       <c r="B29" s="24" t="s">
         <v>93</v>
       </c>
-      <c r="C29" s="8"/>
-      <c r="D29" s="8"/>
-      <c r="E29" s="25"/>
+      <c r="C29" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="E29" s="25" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="23">
         <v>29</v>
       </c>
       <c r="B30" s="24" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C30" s="8"/>
-      <c r="D30" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="E30" s="25" t="s">
-        <v>95</v>
-      </c>
+      <c r="D30" s="8"/>
+      <c r="E30" s="25"/>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="23">
@@ -2549,7 +2537,7 @@
       <c r="D31" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="E31" s="34" t="s">
+      <c r="E31" s="25" t="s">
         <v>97</v>
       </c>
     </row>
@@ -2560,13 +2548,11 @@
       <c r="B32" s="24" t="s">
         <v>98</v>
       </c>
-      <c r="C32" s="8" t="s">
-        <v>43</v>
-      </c>
+      <c r="C32" s="8"/>
       <c r="D32" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="E32" s="34" t="s">
+      <c r="E32" s="33" t="s">
         <v>99</v>
       </c>
     </row>
@@ -2578,12 +2564,12 @@
         <v>100</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>76</v>
+        <v>43</v>
       </c>
       <c r="D33" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="E33" s="34" t="s">
+      <c r="E33" s="33" t="s">
         <v>101</v>
       </c>
     </row>
@@ -2591,10 +2577,18 @@
       <c r="A34" s="23">
         <v>33</v>
       </c>
-      <c r="B34" s="24"/>
-      <c r="C34" s="8"/>
-      <c r="D34" s="8"/>
-      <c r="E34" s="34"/>
+      <c r="B34" s="24" t="s">
+        <v>102</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="E34" s="33" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="23">
@@ -2603,7 +2597,16 @@
       <c r="B35" s="24"/>
       <c r="C35" s="8"/>
       <c r="D35" s="8"/>
-      <c r="E35" s="25"/>
+      <c r="E35" s="33"/>
+    </row>
+    <row r="36" ht="18.15" spans="1:5">
+      <c r="A36" s="27">
+        <v>35</v>
+      </c>
+      <c r="B36" s="28"/>
+      <c r="C36" s="29"/>
+      <c r="D36" s="29"/>
+      <c r="E36" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2643,207 +2646,207 @@
         <v>37</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="39" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C2" s="21"/>
       <c r="D2" s="22" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="40" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="24" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C3" s="8"/>
       <c r="D3" s="25" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="40" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="24" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C4" s="8"/>
       <c r="D4" s="25" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="40" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D5" s="25" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:4">
-      <c r="A6" s="41" t="s">
+      <c r="A6" s="40" t="s">
         <v>14</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D6" s="25" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7" spans="1:4">
-      <c r="A7" s="41" t="s">
+      <c r="A7" s="40" t="s">
         <v>17</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D7" s="25" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="8" spans="1:4">
-      <c r="A8" s="41" t="s">
+      <c r="A8" s="40" t="s">
         <v>20</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C8" s="8"/>
       <c r="D8" s="25" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9" spans="1:4">
-      <c r="A9" s="41" t="s">
+      <c r="A9" s="40" t="s">
         <v>23</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D9" s="25" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10" spans="1:4">
-      <c r="A10" s="41" t="s">
+      <c r="A10" s="40" t="s">
         <v>26</v>
       </c>
       <c r="B10" s="24" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C10" s="8"/>
       <c r="D10" s="26" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="11" spans="1:4">
-      <c r="A11" s="41" t="s">
+      <c r="A11" s="40" t="s">
         <v>29</v>
       </c>
       <c r="B11" s="24" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C11" s="8"/>
       <c r="D11" s="25" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" spans="1:4">
-      <c r="A12" s="41" t="s">
+      <c r="A12" s="40" t="s">
         <v>32</v>
       </c>
       <c r="B12" s="24" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D12" s="25" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="13" spans="1:4">
-      <c r="A13" s="41" t="s">
-        <v>60</v>
+      <c r="A13" s="40" t="s">
+        <v>62</v>
       </c>
       <c r="B13" s="24" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C13" s="8"/>
       <c r="D13" s="25" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:4">
-      <c r="A14" s="41" t="s">
-        <v>61</v>
+      <c r="A14" s="40" t="s">
+        <v>63</v>
       </c>
       <c r="B14" s="24" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C14" s="8"/>
       <c r="D14" s="25" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="15" spans="1:4">
-      <c r="A15" s="41" t="s">
-        <v>63</v>
+      <c r="A15" s="40" t="s">
+        <v>64</v>
       </c>
       <c r="B15" s="24" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C15" s="8"/>
       <c r="D15" s="25" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="16" spans="1:4">
-      <c r="A16" s="41" t="s">
-        <v>65</v>
+      <c r="A16" s="40" t="s">
+        <v>66</v>
       </c>
       <c r="B16" s="24" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C16" s="8"/>
       <c r="D16" s="25"/>
     </row>
     <row r="17" spans="1:4">
-      <c r="A17" s="41" t="s">
+      <c r="A17" s="40" t="s">
         <v>68</v>
       </c>
       <c r="B17" s="24" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C17" s="8"/>
       <c r="D17" s="25" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -2855,7 +2858,7 @@
       </c>
       <c r="C18" s="8"/>
       <c r="D18" s="25" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19" ht="18.15" spans="1:4">
@@ -2863,11 +2866,11 @@
         <v>18</v>
       </c>
       <c r="B19" s="28" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C19" s="29"/>
       <c r="D19" s="30" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -2889,18 +2892,18 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1" spans="1:8">
       <c r="A1" s="11" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D1" s="5"/>
       <c r="E1" s="4"/>
       <c r="F1" s="11" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G1" s="5"/>
       <c r="H1" s="4"/>
@@ -2909,54 +2912,54 @@
       <c r="A2" s="10"/>
       <c r="B2" s="10"/>
       <c r="C2" s="11" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="E2" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="F2" s="11" t="s">
         <v>144</v>
       </c>
-      <c r="F2" s="11" t="s">
-        <v>142</v>
-      </c>
       <c r="G2" s="11" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" ht="16.5" customHeight="1" spans="1:8">
       <c r="A3" s="12" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D3" s="13">
         <v>100</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G3" s="13">
         <v>100</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" ht="16.5" customHeight="1" spans="1:8">
       <c r="A4" s="9"/>
       <c r="B4" s="12" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
@@ -2968,7 +2971,7 @@
     <row r="5" ht="16.5" customHeight="1" spans="1:8">
       <c r="A5" s="9"/>
       <c r="B5" s="12" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
@@ -2980,7 +2983,7 @@
     <row r="6" ht="16.5" customHeight="1" spans="1:8">
       <c r="A6" s="9"/>
       <c r="B6" s="12" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
@@ -2992,7 +2995,7 @@
     <row r="7" ht="16.5" customHeight="1" spans="1:8">
       <c r="A7" s="10"/>
       <c r="B7" s="12" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C7" s="13"/>
       <c r="D7" s="13"/>
@@ -3003,10 +3006,10 @@
     </row>
     <row r="8" ht="16.5" customHeight="1" spans="1:8">
       <c r="A8" s="12" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C8" s="13"/>
       <c r="D8" s="13"/>
@@ -3018,7 +3021,7 @@
     <row r="9" ht="16.5" customHeight="1" spans="1:8">
       <c r="A9" s="9"/>
       <c r="B9" s="12" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
@@ -3030,7 +3033,7 @@
     <row r="10" ht="16.5" customHeight="1" spans="1:8">
       <c r="A10" s="10"/>
       <c r="B10" s="12" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
@@ -3041,10 +3044,10 @@
     </row>
     <row r="11" ht="16.5" customHeight="1" spans="1:8">
       <c r="A11" s="12" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
@@ -3056,7 +3059,7 @@
     <row r="12" ht="16.5" customHeight="1" spans="1:8">
       <c r="A12" s="10"/>
       <c r="B12" s="12" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C12" s="13"/>
       <c r="D12" s="13"/>
@@ -3067,19 +3070,19 @@
     </row>
     <row r="13" ht="16.5" customHeight="1" spans="1:8">
       <c r="A13" s="12" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
@@ -3088,16 +3091,16 @@
     <row r="14" ht="16.5" customHeight="1" spans="1:8">
       <c r="A14" s="10"/>
       <c r="B14" s="12" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>106</v>
-      </c>
-      <c r="D14" s="13" t="s">
-        <v>106</v>
+        <v>108</v>
+      </c>
+      <c r="D14" s="13">
+        <v>100</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>106</v>
+        <v>124</v>
       </c>
       <c r="F14" s="13"/>
       <c r="G14" s="13"/>
@@ -3136,7 +3139,7 @@
   <sheetData>
     <row r="1" ht="16.5" customHeight="1" spans="1:7">
       <c r="A1" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="3" t="s">
@@ -3149,31 +3152,31 @@
     </row>
     <row r="2" ht="16.5" customHeight="1" spans="1:7">
       <c r="A2" s="3" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="3" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="3" ht="16.5" customHeight="1" spans="1:7">
       <c r="A3" s="6" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C3" s="8"/>
       <c r="D3" s="8"/>
@@ -3184,7 +3187,7 @@
     <row r="4" ht="16.5" customHeight="1" spans="1:7">
       <c r="A4" s="9"/>
       <c r="B4" s="7" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C4" s="8"/>
       <c r="D4" s="8"/>
@@ -3195,7 +3198,7 @@
     <row r="5" ht="16.5" customHeight="1" spans="1:7">
       <c r="A5" s="10"/>
       <c r="B5" s="7" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
@@ -3205,10 +3208,10 @@
     </row>
     <row r="6" ht="16.5" customHeight="1" spans="1:7">
       <c r="A6" s="6" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>
@@ -3219,7 +3222,7 @@
     <row r="7" ht="16.5" customHeight="1" spans="1:7">
       <c r="A7" s="9"/>
       <c r="B7" s="7" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
@@ -3230,7 +3233,7 @@
     <row r="8" ht="16.5" customHeight="1" spans="1:7">
       <c r="A8" s="10"/>
       <c r="B8" s="7" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
@@ -3240,10 +3243,10 @@
     </row>
     <row r="9" ht="16.5" customHeight="1" spans="1:7">
       <c r="A9" s="6" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
@@ -3254,7 +3257,7 @@
     <row r="10" ht="16.5" customHeight="1" spans="1:7">
       <c r="A10" s="9"/>
       <c r="B10" s="7" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C10" s="8"/>
       <c r="D10" s="8"/>
@@ -3265,7 +3268,7 @@
     <row r="11" ht="16.5" customHeight="1" spans="1:7">
       <c r="A11" s="10"/>
       <c r="B11" s="7" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C11" s="8"/>
       <c r="D11" s="8"/>
@@ -3275,10 +3278,10 @@
     </row>
     <row r="12" ht="16.5" customHeight="1" spans="1:7">
       <c r="A12" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>
@@ -3289,7 +3292,7 @@
     <row r="13" ht="16.5" customHeight="1" spans="1:7">
       <c r="A13" s="9"/>
       <c r="B13" s="7" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C13" s="8"/>
       <c r="D13" s="8"/>
@@ -3300,7 +3303,7 @@
     <row r="14" ht="16.5" customHeight="1" spans="1:7">
       <c r="A14" s="10"/>
       <c r="B14" s="7" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C14" s="8"/>
       <c r="D14" s="8"/>

</xml_diff>